<commit_message>
add checkout test scripts
</commit_message>
<xml_diff>
--- a/Bug_Reports_saucedemo.xlsx
+++ b/Bug_Reports_saucedemo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Technical Assessment - Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A553ED3-3BE1-493B-BB3A-DB1D3A0F73D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101CC4CA-71CC-4E09-AB34-3195D71646D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FE048FD7-43B9-43C6-893D-01E9F335D6BD}"/>
   </bookViews>
@@ -39,12 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
   <si>
     <t>Bug ID</t>
-  </si>
-  <si>
-    <t>Description</t>
   </si>
   <si>
     <t>Steps to Reproduce</t>
@@ -138,12 +135,6 @@
     <t>System should allow independent input in each field without affecting other fields.</t>
   </si>
   <si>
-    <t>01.Navigate to swag lab login page.
-02. Log in as a problem_user
-03.Click filter drop down menu on inventory ui
-04.Select Price(High to low)</t>
-  </si>
-  <si>
     <t xml:space="preserve">
 01.Navigate to swag lab login page.
 02. Log in as a problem_user
@@ -151,27 +142,20 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">
-01.Navigate to swag lab login page.
-02. Log in as a problem_user.
-03. Click the "Remove" button to remove items from cart.
-</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">System displays abnormal behavior when </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">entering text in the Last Name field. 
-</t>
-    </r>
+    <t>Item total is not rounded.This doesn’t happen when ,
+$10.50 + $5.25 = $15.75</t>
+  </si>
+  <si>
+    <t>System should calculate total price 
+correctly  with tax. And should rounded to two decimal places.
+The Item total should display exactly: Item total: $59.98</t>
+  </si>
+  <si>
+    <t>01.Navigate to swag lab login page.
+02. Log in as a problem_user
+03.Click filter drop down menu on inventory ui
+04.Select Price(High to low).
+05.Observe items order</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -181,44 +165,55 @@
 04.Click "Checkout"
 05.Enter valid First Name
 06.Enter valid Last Name
-07.Enter letter in  Zip/Postal code field</t>
-  </si>
-  <si>
-    <t>Item total is not rounded.This doesn’t happen when ,
-$10.50 + $5.25 = $15.75</t>
+07.View behaviour of the form</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Add to Cart button non-functional for problem_user</t>
+  </si>
+  <si>
+    <t>Remove from Cart button non-functional for problem_user</t>
+  </si>
+  <si>
+    <t>Last Name field input overwrites First Name field for problem_user</t>
+  </si>
+  <si>
+    <t>Item total displays rounding to two decimal point error on Checkout Overview for visual_user</t>
+  </si>
+  <si>
+    <t>Price sort filter fails to apply for problem_user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+01.Navigate to swag lab login page.
+02. Log in as a problem_user.
+03.Click "Add to cart" for some items
+04. Click the "Remove" button to remove those items from the cart.
+</t>
   </si>
   <si>
     <t xml:space="preserve">01.Navigate to swag lab login page.
-02. Log in as a visualize_user.
+02. Log in as a visual_user.
 03.Add the Sauce Labs Bike Light ($9.99) to the cart.
 04.Add the Sauce Labs Fleece Jacket ($49.99) to the cart.
-04.Click "Checkout".Checkout button is on top rightside of the ui
-05.Enter valid First Name
-06.Enter valid Last Name
-07.Enter letter in  Zip/Postal code field
-08.Click "Continue" on Your information ui
-09.View overview page
-10.Observe the calculated "Item total".
+05.Click cart icon.
+06.Click "Checkout".Checkout button is on top rightside of the ui
+07.Enter valid First Name
+08.Enter valid Last Name
+09.Enter valid   Zip/Postal code
+10.Click "Continue" on Your information ui
+11.View overview page
+12.Observe the calculated "Item total".
 </t>
-  </si>
-  <si>
-    <t>System should calculate total price 
-correctly  with tax. And should rounded to two decimal places.
-The Item total should display exactly: Item total: $59.98</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Price(High to low) Option not getting selected.Items are not sorted correctly 
-from high price to low prices.</t>
-  </si>
-  <si>
-    <t>When there are already items on the cart.Those items canot be removed from the cart, and the buttons appear to be frozen.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -260,13 +255,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -546,7 +534,7 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>76200</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -577,8 +565,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14688967" y="8753554"/>
-          <a:ext cx="6384112" cy="3624272"/>
+          <a:off x="14782800" y="8763000"/>
+          <a:ext cx="6321294" cy="3622698"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -590,7 +578,7 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>7872</xdr:colOff>
+      <xdr:colOff>19050</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>7872</xdr:rowOff>
     </xdr:from>
@@ -621,8 +609,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14696839" y="12382500"/>
-          <a:ext cx="6360496" cy="3009195"/>
+          <a:off x="14725650" y="12390372"/>
+          <a:ext cx="6363074" cy="3009195"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1053,152 +1041,152 @@
   <sheetData>
     <row r="7" spans="1:10" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="4" t="s">
-        <v>5</v>
-      </c>
       <c r="H7" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I7" s="5"/>
     </row>
     <row r="8" spans="1:10" ht="285" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:10" ht="285" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H9" s="2"/>
     </row>
     <row r="10" spans="1:10" ht="285" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:10" ht="285" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="11" t="s">
-        <v>33</v>
-      </c>
       <c r="E11" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:10" ht="285" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H12" s="2"/>
       <c r="J12" s="12" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>